<commit_message>
fix(contracts): require explicit competing death dates
</commit_message>
<xml_diff>
--- a/data/fixtures/partner_messy/partner_messy.xlsx
+++ b/data/fixtures/partner_messy/partner_messy.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>days_to_death</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>index_day</t>
         </is>
       </c>
@@ -474,6 +479,9 @@
         <v>1222</v>
       </c>
       <c r="F2" t="n">
+        <v>1222</v>
+      </c>
+      <c r="G2" t="n">
         <v>188</v>
       </c>
     </row>
@@ -499,7 +507,7 @@
       <c r="E3" t="n">
         <v>1231</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>243</v>
       </c>
     </row>
@@ -523,6 +531,9 @@
         <v>1787</v>
       </c>
       <c r="F4" t="n">
+        <v>1787</v>
+      </c>
+      <c r="G4" t="n">
         <v>293</v>
       </c>
     </row>
@@ -548,7 +559,7 @@
       <c r="E5" t="n">
         <v>2254</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>63</v>
       </c>
     </row>
@@ -575,6 +586,9 @@
         <v>433</v>
       </c>
       <c r="F6" t="n">
+        <v>433</v>
+      </c>
+      <c r="G6" t="n">
         <v>177</v>
       </c>
     </row>
@@ -600,7 +614,7 @@
       <c r="E7" t="n">
         <v>2603</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>259</v>
       </c>
     </row>
@@ -626,7 +640,7 @@
       <c r="E8" t="n">
         <v>504</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>261</v>
       </c>
     </row>
@@ -653,6 +667,9 @@
         <v>2844</v>
       </c>
       <c r="F9" t="n">
+        <v>2844</v>
+      </c>
+      <c r="G9" t="n">
         <v>133</v>
       </c>
     </row>
@@ -678,7 +695,7 @@
       <c r="E10" t="n">
         <v>882</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>275</v>
       </c>
     </row>
@@ -704,7 +721,7 @@
       <c r="E11" t="n">
         <v>2238</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>150</v>
       </c>
     </row>
@@ -730,7 +747,7 @@
       <c r="E12" t="n">
         <v>995</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>179</v>
       </c>
     </row>
@@ -756,7 +773,7 @@
       <c r="E13" t="n">
         <v>1784</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>205</v>
       </c>
     </row>
@@ -782,7 +799,7 @@
       <c r="E14" t="n">
         <v>1856</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>200</v>
       </c>
     </row>
@@ -808,7 +825,7 @@
       <c r="E15" t="n">
         <v>599</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>266</v>
       </c>
     </row>
@@ -836,7 +853,7 @@
           <t>ten</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>221</v>
       </c>
     </row>
@@ -862,7 +879,7 @@
       <c r="E17" t="n">
         <v>2438</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>108</v>
       </c>
     </row>
@@ -888,7 +905,7 @@
       <c r="E18" t="n">
         <v>1071</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>179</v>
       </c>
     </row>
@@ -915,6 +932,9 @@
         <v>1976</v>
       </c>
       <c r="F19" t="n">
+        <v>1976</v>
+      </c>
+      <c r="G19" t="n">
         <v>2026</v>
       </c>
     </row>
@@ -940,7 +960,7 @@
       <c r="E20" t="n">
         <v>1528</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>162</v>
       </c>
     </row>
@@ -966,7 +986,7 @@
       <c r="E21" t="n">
         <v>434</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>76</v>
       </c>
     </row>
@@ -992,7 +1012,7 @@
       <c r="E22" t="n">
         <v>976</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>144</v>
       </c>
     </row>
@@ -1018,7 +1038,7 @@
       <c r="E23" t="n">
         <v>693</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>153</v>
       </c>
     </row>
@@ -1044,7 +1064,7 @@
       <c r="E24" t="n">
         <v>1767</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>180</v>
       </c>
     </row>
@@ -1070,7 +1090,7 @@
       <c r="E25" t="n">
         <v>1218</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>180</v>
       </c>
     </row>
@@ -1096,7 +1116,7 @@
       <c r="E26" t="n">
         <v>713</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>225</v>
       </c>
     </row>
@@ -1123,6 +1143,9 @@
         <v>2794</v>
       </c>
       <c r="F27" t="n">
+        <v>2794</v>
+      </c>
+      <c r="G27" t="n">
         <v>96</v>
       </c>
     </row>
@@ -1148,7 +1171,7 @@
       <c r="E28" t="n">
         <v>973</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>289</v>
       </c>
     </row>
@@ -1174,7 +1197,7 @@
       <c r="E29" t="n">
         <v>2791</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>105</v>
       </c>
     </row>
@@ -1200,7 +1223,7 @@
       <c r="E30" t="n">
         <v>2487</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>109</v>
       </c>
     </row>
@@ -1226,7 +1249,7 @@
       <c r="E31" t="n">
         <v>2506</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>128</v>
       </c>
     </row>
@@ -1252,7 +1275,7 @@
       <c r="E32" t="n">
         <v>1541</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>276</v>
       </c>
     </row>
@@ -1278,7 +1301,7 @@
       <c r="E33" t="n">
         <v>2574</v>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>165</v>
       </c>
     </row>
@@ -1304,7 +1327,7 @@
       <c r="E34" t="n">
         <v>2317</v>
       </c>
-      <c r="F34" t="n">
+      <c r="G34" t="n">
         <v>299</v>
       </c>
     </row>
@@ -1331,6 +1354,9 @@
         <v>2327</v>
       </c>
       <c r="F35" t="n">
+        <v>2327</v>
+      </c>
+      <c r="G35" t="n">
         <v>280</v>
       </c>
     </row>
@@ -1356,7 +1382,7 @@
       <c r="E36" t="n">
         <v>809</v>
       </c>
-      <c r="F36" t="n">
+      <c r="G36" t="n">
         <v>127</v>
       </c>
     </row>
@@ -1382,7 +1408,7 @@
       <c r="E37" t="n">
         <v>527</v>
       </c>
-      <c r="F37" t="n">
+      <c r="G37" t="n">
         <v>224</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="E38" t="n">
         <v>2389</v>
       </c>
-      <c r="F38" t="n">
+      <c r="G38" t="n">
         <v>181</v>
       </c>
     </row>
@@ -1435,6 +1461,9 @@
         <v>1986</v>
       </c>
       <c r="F39" t="n">
+        <v>1986</v>
+      </c>
+      <c r="G39" t="n">
         <v>245</v>
       </c>
     </row>
@@ -1460,7 +1489,7 @@
       <c r="E40" t="n">
         <v>2445</v>
       </c>
-      <c r="F40" t="n">
+      <c r="G40" t="n">
         <v>258</v>
       </c>
     </row>
@@ -1487,6 +1516,9 @@
         <v>1041</v>
       </c>
       <c r="F41" t="n">
+        <v>1041</v>
+      </c>
+      <c r="G41" t="n">
         <v>156</v>
       </c>
     </row>
@@ -1512,7 +1544,7 @@
       <c r="E42" t="n">
         <v>1983</v>
       </c>
-      <c r="F42" t="n">
+      <c r="G42" t="n">
         <v>145</v>
       </c>
     </row>
@@ -1538,7 +1570,7 @@
       <c r="E43" t="n">
         <v>722</v>
       </c>
-      <c r="F43" t="n">
+      <c r="G43" t="n">
         <v>162</v>
       </c>
     </row>
@@ -1564,7 +1596,7 @@
       <c r="E44" t="n">
         <v>1629</v>
       </c>
-      <c r="F44" t="n">
+      <c r="G44" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1590,7 +1622,7 @@
       <c r="E45" t="n">
         <v>2112</v>
       </c>
-      <c r="F45" t="n">
+      <c r="G45" t="n">
         <v>134</v>
       </c>
     </row>
@@ -1617,6 +1649,9 @@
         <v>2892</v>
       </c>
       <c r="F46" t="n">
+        <v>2892</v>
+      </c>
+      <c r="G46" t="n">
         <v>294</v>
       </c>
     </row>
@@ -1642,7 +1677,7 @@
       <c r="E47" t="n">
         <v>2294</v>
       </c>
-      <c r="F47" t="n">
+      <c r="G47" t="n">
         <v>262</v>
       </c>
     </row>
@@ -1668,7 +1703,7 @@
       <c r="E48" t="n">
         <v>2430</v>
       </c>
-      <c r="F48" t="n">
+      <c r="G48" t="n">
         <v>82</v>
       </c>
     </row>
@@ -1694,7 +1729,7 @@
       <c r="E49" t="n">
         <v>930</v>
       </c>
-      <c r="F49" t="n">
+      <c r="G49" t="n">
         <v>161</v>
       </c>
     </row>
@@ -1720,7 +1755,7 @@
       <c r="E50" t="n">
         <v>2656</v>
       </c>
-      <c r="F50" t="n">
+      <c r="G50" t="n">
         <v>235</v>
       </c>
     </row>
@@ -1746,7 +1781,7 @@
       <c r="E51" t="n">
         <v>1025</v>
       </c>
-      <c r="F51" t="n">
+      <c r="G51" t="n">
         <v>178</v>
       </c>
     </row>
@@ -1772,7 +1807,7 @@
       <c r="E52" t="n">
         <v>2881</v>
       </c>
-      <c r="F52" t="n">
+      <c r="G52" t="n">
         <v>145</v>
       </c>
     </row>
@@ -1799,6 +1834,9 @@
         <v>553</v>
       </c>
       <c r="F53" t="n">
+        <v>553</v>
+      </c>
+      <c r="G53" t="n">
         <v>263</v>
       </c>
     </row>
@@ -1824,7 +1862,7 @@
       <c r="E54" t="n">
         <v>936</v>
       </c>
-      <c r="F54" t="n">
+      <c r="G54" t="n">
         <v>255</v>
       </c>
     </row>
@@ -1851,6 +1889,9 @@
         <v>2042</v>
       </c>
       <c r="F55" t="n">
+        <v>2042</v>
+      </c>
+      <c r="G55" t="n">
         <v>150</v>
       </c>
     </row>
@@ -1876,7 +1917,7 @@
       <c r="E56" t="n">
         <v>1776</v>
       </c>
-      <c r="F56" t="n">
+      <c r="G56" t="n">
         <v>195</v>
       </c>
     </row>
@@ -1902,7 +1943,7 @@
       <c r="E57" t="n">
         <v>1848</v>
       </c>
-      <c r="F57" t="n">
+      <c r="G57" t="n">
         <v>74</v>
       </c>
     </row>
@@ -1928,7 +1969,7 @@
       <c r="E58" t="n">
         <v>734</v>
       </c>
-      <c r="F58" t="n">
+      <c r="G58" t="n">
         <v>218</v>
       </c>
     </row>
@@ -1955,6 +1996,9 @@
         <v>1931</v>
       </c>
       <c r="F59" t="n">
+        <v>1931</v>
+      </c>
+      <c r="G59" t="n">
         <v>242</v>
       </c>
     </row>
@@ -1980,7 +2024,7 @@
       <c r="E60" t="n">
         <v>1247</v>
       </c>
-      <c r="F60" t="n">
+      <c r="G60" t="n">
         <v>102</v>
       </c>
     </row>
@@ -2007,6 +2051,9 @@
         <v>1245</v>
       </c>
       <c r="F61" t="n">
+        <v>1245</v>
+      </c>
+      <c r="G61" t="n">
         <v>276</v>
       </c>
     </row>
@@ -2032,7 +2079,7 @@
       <c r="E62" t="n">
         <v>1784</v>
       </c>
-      <c r="F62" t="n">
+      <c r="G62" t="n">
         <v>205</v>
       </c>
     </row>

</xml_diff>